<commit_message>
Redesign: 3-layer data model (Master+batch+manual), bulk+single modes
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FD_Renewal" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UT_Subscription" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UT_Redemption" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UT_Switch" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,31 +429,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ic_number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>ic_number</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -501,57 +505,537 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>880101-14-5678</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>TAN AH KAW</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>012-3456789</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>tan@email.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No. 12, Jalan Maju</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Taman Indah</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>WP KL</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>01/01/1988</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>901215-08-1234</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LIM VOON SIM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>016-7654321</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>lim@email.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No. 5, Jalan Damai</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Petaling Jaya</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Selangor</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>47500</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>15/12/1990</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Accountant</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>750320-05-9876</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WONG MEI LING</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>011-2233445</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>wong@email.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No. 88, Lorong Bahagia</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Taman Sejahtera</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Johor Bahru</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Johor</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>80100</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>20/03/1975</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Business Owner</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ic_number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>fd_account_no</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>fd_amount</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>maturity_date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>renewal_period</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>interest_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>880101-14-5678</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>2141-00012345</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>3.55%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>901215-08-1234</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2141-00098765</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>6 months</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3.60%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ic_number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>fund_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>payment_method</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ut_account_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>880101-14-5678</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RHB Global AI Fund</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>012-3456789</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>tan@email.com</t>
+          <t>Online Transfer</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>No. 12, Jalan Maju</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Taman Indah</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Kuala Lumpur</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Wilayah Persekutuan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>50000</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>01/01/1988</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Engineer</t>
+          <t>8-12116-0000001-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>750320-05-9876</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RHB Dynamic AI Allocator</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cheque</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8-12116-0000002-3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ic_number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>fund_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>bank_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>bank_account_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>901215-08-1234</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RHB Global AI Fund</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1500.00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1234-5678-9012</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ic_number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>switch_out_fund</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>switch_in_fund</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ut_account_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>880101-14-5678</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RHB Bond Fund</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RHB Global AI Fund</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2000.00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>8-12116-0000001-1</t>
         </is>
       </c>
     </row>

</xml_diff>